<commit_message>
Corrige Resumo: frequência agregada em vez de média de percentuais
Cálculo anterior: média dos % por pergunta (média de médias).
Cálculo novo: soma de respostas positivas ÷ total de respostas válidas
na esfera × grupo (frequência pooled). Denominador exclui não-respostas.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YaN6iQfVUePBZHakcrumrR
</commit_message>
<xml_diff>
--- a/analise_frequencia_por_grupo.xlsx
+++ b/analise_frequencia_por_grupo.xlsx
@@ -24,7 +24,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -95,8 +95,22 @@
       <color rgb="00666666"/>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00333333"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -148,8 +162,13 @@
         <fgColor rgb="00F5F5F5"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -171,11 +190,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -250,6 +283,24 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="11" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -615,367 +666,416 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Resumo — % Concordância e Participação por Grupo de Autoposicionamento (Q10)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="B2" s="2" t="inlineStr">
+          <t>Resumo — % Frequência Agregada por Grupo de Autoposicionamento (Q10)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="30" t="inlineStr">
+        <is>
+          <t>Cálculo: soma das respostas positivas (Sim / Concordo / Participa) ÷ total de respostas válidas na esfera para o grupo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="16" customHeight="1">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>N = 20</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>N = 13</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>N = 13</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>N = 51</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>N = 28</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>N = 6</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>N = 10</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Esfera / Indicador</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>Novo</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>Adaptando</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>Inserindo</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E4" s="4" t="inlineStr">
         <is>
           <t>Comprometido</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Ativo No Motivo</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>Embaixador</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>Cocriador</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>Conhecimento Institucional — % Sim (média 4 perguntas)</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="n">
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="31" t="inlineStr">
+        <is>
+          <t>Conhecimento Institucional — % Sim</t>
+        </is>
+      </c>
+      <c r="B5" s="32" t="n">
         <v>0.6</v>
       </c>
-      <c r="C4" s="6" t="n">
-        <v>0.7114999999999999</v>
-      </c>
-      <c r="D4" s="6" t="n">
-        <v>0.5575</v>
-      </c>
-      <c r="E4" s="6" t="n">
-        <v>0.72075</v>
-      </c>
-      <c r="F4" s="6" t="n">
+      <c r="C5" s="32" t="n">
+        <v>0.7115384615384616</v>
+      </c>
+      <c r="D5" s="32" t="n">
+        <v>0.5576923076923077</v>
+      </c>
+      <c r="E5" s="32" t="n">
+        <v>0.7241379310344828</v>
+      </c>
+      <c r="F5" s="32" t="n">
         <v>0.8125</v>
       </c>
-      <c r="G4" s="6" t="n">
-        <v>0.95825</v>
-      </c>
-      <c r="H4" s="6" t="n">
+      <c r="G5" s="32" t="n">
+        <v>0.9583333333333334</v>
+      </c>
+      <c r="H5" s="32" t="n">
         <v>0.85</v>
       </c>
     </row>
-    <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>Pertencimento Cultural — % Concorda (total, média)</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="n">
+    <row r="6" ht="13" customHeight="1">
+      <c r="A6" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     ↳ Perguntas 4, 5, 6 e 9 (Sim/Não)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="31" t="inlineStr">
+        <is>
+          <t>Pertencimento Cultural — % Concorda (total)</t>
+        </is>
+      </c>
+      <c r="B7" s="32" t="n">
         <v>0.95625</v>
       </c>
-      <c r="C5" s="6" t="n">
-        <v>0.9807499999999999</v>
-      </c>
-      <c r="D5" s="6" t="n">
-        <v>0.9614999999999999</v>
-      </c>
-      <c r="E5" s="6" t="n">
-        <v>0.990125</v>
-      </c>
-      <c r="F5" s="6" t="n">
+      <c r="C7" s="32" t="n">
+        <v>0.9807692307692307</v>
+      </c>
+      <c r="D7" s="32" t="n">
+        <v>0.9615384615384616</v>
+      </c>
+      <c r="E7" s="32" t="n">
+        <v>0.9901960784313726</v>
+      </c>
+      <c r="F7" s="32" t="n">
         <v>1</v>
       </c>
-      <c r="G5" s="6" t="n">
+      <c r="G7" s="32" t="n">
         <v>1</v>
       </c>
-      <c r="H5" s="6" t="n">
+      <c r="H7" s="32" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Concordo (pleno)</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="n">
+    <row r="8" ht="13" customHeight="1">
+      <c r="A8" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     ↳ 8 afirmações — Concordo + Concordo parcialmente</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Concordo pleno</t>
+        </is>
+      </c>
+      <c r="B9" s="35" t="n">
         <v>0.85625</v>
       </c>
-      <c r="C6" s="8" t="n">
-        <v>0.82675</v>
-      </c>
-      <c r="D6" s="8" t="n">
-        <v>0.6729999999999999</v>
-      </c>
-      <c r="E6" s="8" t="n">
-        <v>0.9214999999999999</v>
-      </c>
-      <c r="F6" s="8" t="n">
-        <v>0.857125</v>
-      </c>
-      <c r="G6" s="8" t="n">
-        <v>0.937375</v>
-      </c>
-      <c r="H6" s="8" t="n">
+      <c r="C9" s="35" t="n">
+        <v>0.8269230769230769</v>
+      </c>
+      <c r="D9" s="35" t="n">
+        <v>0.6730769230769231</v>
+      </c>
+      <c r="E9" s="35" t="n">
+        <v>0.9215686274509803</v>
+      </c>
+      <c r="F9" s="35" t="n">
+        <v>0.8571428571428571</v>
+      </c>
+      <c r="G9" s="35" t="n">
+        <v>0.9375</v>
+      </c>
+      <c r="H9" s="35" t="n">
         <v>0.8625</v>
       </c>
     </row>
-    <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Acordos Sociais — % Concorda (total, média)</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="n">
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="31" t="inlineStr">
+        <is>
+          <t>Acordos Sociais — % Concorda (total)</t>
+        </is>
+      </c>
+      <c r="B10" s="32" t="n">
         <v>0.5388888888888889</v>
       </c>
-      <c r="C7" s="6" t="n">
-        <v>0.7691111111111111</v>
-      </c>
-      <c r="D7" s="6" t="n">
-        <v>0.8631111111111109</v>
-      </c>
-      <c r="E7" s="6" t="n">
-        <v>0.9127777777777779</v>
-      </c>
-      <c r="F7" s="6" t="n">
-        <v>0.9603333333333335</v>
-      </c>
-      <c r="G7" s="6" t="n">
-        <v>0.9443333333333332</v>
-      </c>
-      <c r="H7" s="6" t="n">
+      <c r="C10" s="32" t="n">
+        <v>0.7692307692307693</v>
+      </c>
+      <c r="D10" s="32" t="n">
+        <v>0.8632478632478633</v>
+      </c>
+      <c r="E10" s="32" t="n">
+        <v>0.9128540305010894</v>
+      </c>
+      <c r="F10" s="32" t="n">
+        <v>0.9603174603174603</v>
+      </c>
+      <c r="G10" s="32" t="n">
+        <v>0.9444444444444444</v>
+      </c>
+      <c r="H10" s="32" t="n">
         <v>0.9777777777777777</v>
       </c>
     </row>
-    <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Concordo (pleno)</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="n">
+    <row r="11" ht="13" customHeight="1">
+      <c r="A11" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     ↳ 9 afirmações — Concordo + Concordo parcialmente</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Concordo pleno</t>
+        </is>
+      </c>
+      <c r="B12" s="35" t="n">
         <v>0.4722222222222222</v>
       </c>
-      <c r="C8" s="8" t="n">
-        <v>0.3933333333333334</v>
-      </c>
-      <c r="D8" s="8" t="n">
-        <v>0.4786666666666667</v>
-      </c>
-      <c r="E8" s="8" t="n">
-        <v>0.7581111111111111</v>
-      </c>
-      <c r="F8" s="8" t="n">
+      <c r="C12" s="35" t="n">
+        <v>0.3931623931623932</v>
+      </c>
+      <c r="D12" s="35" t="n">
+        <v>0.4786324786324787</v>
+      </c>
+      <c r="E12" s="35" t="n">
+        <v>0.7581699346405228</v>
+      </c>
+      <c r="F12" s="35" t="n">
         <v>0.75</v>
       </c>
-      <c r="G8" s="8" t="n">
-        <v>0.685111111111111</v>
-      </c>
-      <c r="H8" s="8" t="n">
+      <c r="G12" s="35" t="n">
+        <v>0.6851851851851852</v>
+      </c>
+      <c r="H12" s="35" t="n">
         <v>0.7</v>
       </c>
     </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Prática da Economia Fraterna — % Concorda (total, média)</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="n">
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="31" t="inlineStr">
+        <is>
+          <t>Economia Fraterna — % Concorda (total)</t>
+        </is>
+      </c>
+      <c r="B13" s="32" t="n">
         <v>0.75</v>
       </c>
-      <c r="C9" s="6" t="n">
-        <v>0.7596250000000001</v>
-      </c>
-      <c r="D9" s="6" t="n">
-        <v>0.7882499999999999</v>
-      </c>
-      <c r="E9" s="6" t="n">
-        <v>0.8921250000000001</v>
-      </c>
-      <c r="F9" s="6" t="n">
-        <v>0.937375</v>
-      </c>
-      <c r="G9" s="6" t="n">
-        <v>0.8122499999999999</v>
-      </c>
-      <c r="H9" s="6" t="n">
+      <c r="C13" s="32" t="n">
+        <v>0.7596153846153846</v>
+      </c>
+      <c r="D13" s="32" t="n">
+        <v>0.7884615384615384</v>
+      </c>
+      <c r="E13" s="32" t="n">
+        <v>0.8921568627450981</v>
+      </c>
+      <c r="F13" s="32" t="n">
         <v>0.9375</v>
       </c>
-    </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Concordo (pleno)</t>
-        </is>
-      </c>
-      <c r="B10" s="8" t="n">
+      <c r="G13" s="32" t="n">
+        <v>0.8125</v>
+      </c>
+      <c r="H13" s="32" t="n">
+        <v>0.9375</v>
+      </c>
+    </row>
+    <row r="14" ht="13" customHeight="1">
+      <c r="A14" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     ↳ 8 afirmações — Concordo + Concordo parcialmente</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Concordo pleno</t>
+        </is>
+      </c>
+      <c r="B15" s="35" t="n">
         <v>0.64375</v>
       </c>
-      <c r="C10" s="8" t="n">
-        <v>0.480625</v>
-      </c>
-      <c r="D10" s="8" t="n">
-        <v>0.308</v>
-      </c>
-      <c r="E10" s="8" t="n">
-        <v>0.68875</v>
-      </c>
-      <c r="F10" s="8" t="n">
-        <v>0.7232500000000001</v>
-      </c>
-      <c r="G10" s="8" t="n">
+      <c r="C15" s="35" t="n">
+        <v>0.4807692307692308</v>
+      </c>
+      <c r="D15" s="35" t="n">
+        <v>0.3076923076923077</v>
+      </c>
+      <c r="E15" s="35" t="n">
+        <v>0.6887254901960784</v>
+      </c>
+      <c r="F15" s="35" t="n">
+        <v>0.7232142857142857</v>
+      </c>
+      <c r="G15" s="35" t="n">
         <v>0.5625</v>
       </c>
-      <c r="H10" s="8" t="n">
+      <c r="H15" s="35" t="n">
         <v>0.6875</v>
       </c>
     </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>Engajamento — % Participa ou já participou (média)</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="n">
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="31" t="inlineStr">
+        <is>
+          <t>Engajamento — % Participa ou já participou</t>
+        </is>
+      </c>
+      <c r="B16" s="32" t="n">
         <v>0.24</v>
       </c>
-      <c r="C11" s="6" t="n">
-        <v>0.3076</v>
-      </c>
-      <c r="D11" s="6" t="n">
-        <v>0.5076000000000001</v>
-      </c>
-      <c r="E11" s="6" t="n">
-        <v>0.5294</v>
-      </c>
-      <c r="F11" s="6" t="n">
-        <v>0.7714</v>
-      </c>
-      <c r="G11" s="6" t="n">
-        <v>0.7665999999999999</v>
-      </c>
-      <c r="H11" s="6" t="n">
+      <c r="C16" s="32" t="n">
+        <v>0.3076923076923077</v>
+      </c>
+      <c r="D16" s="32" t="n">
+        <v>0.5076923076923077</v>
+      </c>
+      <c r="E16" s="32" t="n">
+        <v>0.5294117647058824</v>
+      </c>
+      <c r="F16" s="32" t="n">
+        <v>0.7714285714285715</v>
+      </c>
+      <c r="G16" s="32" t="n">
+        <v>0.7666666666666667</v>
+      </c>
+      <c r="H16" s="32" t="n">
         <v>0.66</v>
       </c>
     </row>
-    <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Sou atualmente (algum papel ativo)</t>
-        </is>
-      </c>
-      <c r="B12" s="8" t="n">
+    <row r="17" ht="13" customHeight="1">
+      <c r="A17" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     ↳ 5 papéis — Sou atualmente + Já fui</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Sou atualmente (papel ativo)</t>
+        </is>
+      </c>
+      <c r="B18" s="35" t="n">
         <v>0.06</v>
       </c>
-      <c r="C12" s="8" t="n">
-        <v>0.0924</v>
-      </c>
-      <c r="D12" s="8" t="n">
-        <v>0.077</v>
-      </c>
-      <c r="E12" s="8" t="n">
-        <v>0.0708</v>
-      </c>
-      <c r="F12" s="8" t="n">
-        <v>0.2786</v>
-      </c>
-      <c r="G12" s="8" t="n">
+      <c r="C18" s="35" t="n">
+        <v>0.09230769230769231</v>
+      </c>
+      <c r="D18" s="35" t="n">
+        <v>0.07692307692307693</v>
+      </c>
+      <c r="E18" s="35" t="n">
+        <v>0.07058823529411765</v>
+      </c>
+      <c r="F18" s="35" t="n">
+        <v>0.2785714285714286</v>
+      </c>
+      <c r="G18" s="35" t="n">
         <v>0.3</v>
       </c>
-      <c r="H12" s="8" t="n">
+      <c r="H18" s="35" t="n">
         <v>0.26</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="9" t="inlineStr">
-        <is>
-          <t>Grupos definidos pela resposta à pergunta 10 (autoposicionamento). N total = 141 respondentes com autoposicionamento válido.</t>
+    <row r="20">
+      <c r="A20" s="33" t="inlineStr">
+        <is>
+          <t>N total = 141 respondentes com autoposicionamento válido (Q10). Respondentes sem resposta em cada pergunta são excluídos do denominador.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="8">
+    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A11:H11"/>
+    <mergeCell ref="A14:H14"/>
     <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="A6:H6"/>
+    <mergeCell ref="A17:H17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1009,8 +1109,6 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
       <c r="C2" s="2" t="inlineStr">
         <is>
           <t>N = 20</t>
@@ -1383,8 +1481,6 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
       <c r="C2" s="2" t="inlineStr">
         <is>
           <t>N = 20</t>
@@ -2744,8 +2840,6 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
       <c r="C2" s="2" t="inlineStr">
         <is>
           <t>N = 20</t>
@@ -4259,8 +4353,6 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
       <c r="C2" s="2" t="inlineStr">
         <is>
           <t>N = 20</t>
@@ -5619,8 +5711,6 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
       <c r="C2" s="2" t="inlineStr">
         <is>
           <t>N = 20</t>

</xml_diff>